<commit_message>
Stage 8 fixes: E-008
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Stability/XA5/WA-2022-226/Results/Approved/XA5_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
+++ b/output/archive/WestravelleData/Stability/XA5/WA-2022-226/Results/Approved/XA5_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
@@ -472,7 +472,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WA/2022/226 XA5 pulls and suitability results</t>
+          <t>Westravelle Analytical Ltd, a Tarnovell company: WA/2022/226 XA5 results</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Complies at all conditions and timepoints; shake-before-use instruction added after resuspension check</t>
+          <t>ICH storage pulls comply; resuspension assessment supported shake-before-use instruction. No eighteen-month opened/reconstituted in-use claim.</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Assay as % label claim, impurities as % area. Water by Karl Fischer, % w/w. Bottles were stored upright and shaken before each withdrawal, as per the protocol.</t>
+          <t>Assay as % label claim, impurities as % area; water by Karl Fischer, % w/w. Timepoint means product age at the ICH storage pull, not elapsed time after reconstitution or opening. Opening/reconstitution histories are in bottle-specific batch cards under WST-22-007025.</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1367,14 +1367,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Resuspension after storage: dosing instruction basis</t>
+          <t>Resuspension assessment: dosing instruction basis</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bottles held at the labelled storage condition were left unshaken for the stated interval, then resuspended by hand before sampling. Observations recorded per bottle.</t>
+          <t>Source: WA/2022/226 resuspension protocol and bottle observation sheets linked from batch card WST-22-007025.</t>
         </is>
       </c>
     </row>
@@ -1382,85 +1382,102 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Record component</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Source / scope</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>Interpretation</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Time to visible sediment</t>
+          <t>Bottle/sample identification</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Sediment within the protocol window</t>
+          <t>Bottle observation sheet and withdrawal sample labels</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Settled, no caking</t>
+          <t>Bottle identifiers are not reproduced here.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Resuspension by inversion</t>
+          <t>Reconstitution/opening date and in-use interval</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Uniform after the labelled number of inversions</t>
+          <t>Bottle preparation entries and protocol-defined interval</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Shake-before-use wording supported</t>
+          <t>Do not substitute ICH product age for in-use interval.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Dose content after resuspension</t>
+          <t>Withdrawal and shaking procedure</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Within the assay limits</t>
+          <t>Protocol instructions and per-bottle execution record: shaking/inversion, settling interval, withdrawal order and sampling position</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Samples taken from top, middle and bottom of the bottle</t>
+          <t>Specific counts, times and repeat-withdrawal history are not transcribed here.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Conclusion</t>
+          <t>Dose-uniformity acceptance</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Shake-before-use instruction added to the label</t>
+          <t>Protocol acceptance criteria and signed dose-content sequence sheets</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Requested by Xarnelvune on 14/03/2024</t>
+          <t>No bottle-specific measured result or independent uniformity acceptance asserted here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Known outcome at issue</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Assessment supported dosing instructions; shake-before-use instruction added</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Recorded at issue 08/02/2024; no later label-request date.</t>
         </is>
       </c>
     </row>

</xml_diff>